<commit_message>
📊 Horarios actualizados Línea 141 - 3996
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:20:32</t>
+          <t>Última actualización: 03:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:20:32</t>
+          <t>03:45:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:58</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:20:32</t>
+          <t>03:45:53</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:03</t>
+          <t>03:51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,234 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>103</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>04:44</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>59</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>62</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:04</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>79</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>92</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>99</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:24</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>99</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:38</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>113</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>117</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>119</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:20:32</t>
+          <t>Última actualización: 03:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -585,12 +810,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:20:32</t>
+          <t>03:45:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:03</t>
+          <t>03:51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,9 +824,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>103</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>62</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05:24</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>99</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -618,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,14 +906,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:20:32</t>
+          <t>Última actualización: 03:45:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>03:45:53</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:33</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>108</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3997
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:53</t>
+          <t>Última actualización: 06:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -740,6 +740,806 @@
         <v>119</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:26</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:33</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>86XR36_ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:43</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>17</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>06:46</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>06:49</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>23</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:52</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>26</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:57</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>31</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:57</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>31</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>38</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>39</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:08</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>42</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>46</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>48</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07:18</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>52</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>55</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>58</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>07:25</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>59</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>60</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>62</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>64</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>65</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>70</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:47</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>81</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>83</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>90</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>97</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:04</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>98</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>08:07</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>101</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:13</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>107</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>113</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>115</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>117</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -769,14 +1569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:53</t>
+          <t>Última actualización: 06:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -877,6 +1677,81 @@
         <v>99</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:43</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>17</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>46</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>62</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -893,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:45:53</t>
+          <t>Última actualización: 06:26:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -964,6 +1839,131 @@
         <v>108</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>19</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:53</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>27</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>61</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>82</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:26:32</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>119</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3998
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:32</t>
+          <t>Última actualización: 08:35:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 72</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1540,6 +1540,731 @@
         <v>117</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>13</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>15</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>17</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>24</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>28</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>29</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>39</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>39</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>41</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>44</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>46</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>55</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>55</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>59</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:37</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>62</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>69</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>70</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>84</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>89</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>91</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>92</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>98</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>105</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>106</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>109</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>110</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1556,7 +2281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1569,14 +2294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:32</t>
+          <t>Última actualización: 08:35:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1752,6 +2477,156 @@
         <v>62</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:35</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>44</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>69</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>89</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:26:32</t>
+          <t>Última actualización: 08:35:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1966,6 +2841,131 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>104</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>107</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3999
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:35:04</t>
+          <t>Última actualización: 10:15:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 72</t>
+          <t>Total filas: 109</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:35:04</t>
+          <t>10:15:20</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>105</v>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:35:04</t>
+          <t>10:15:20</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>10:16</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:35:04</t>
+          <t>10:15:20</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>109</v>
+        <v>3</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2253,18 +2253,943 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>105</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>6</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>9</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>9</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>10:25</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D81" t="n">
         <v>110</v>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>15</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>17</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>19</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>19</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>25</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>29</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>29</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>33</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>10:49</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>34</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>38</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>39</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>43</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>45</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>46</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>49</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>54</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>56</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>58</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>59</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>66</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>66</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>69</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>70</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>74</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>79</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>11:37</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>82</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>85</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>91</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>11:47</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>92</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>97</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>98</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>106</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>12:12</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>117</v>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2281,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2294,14 +3219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:35:04</t>
+          <t>Última actualización: 10:15:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -2627,6 +3552,156 @@
         <v>89</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:16</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>66</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>69</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>91</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>106</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2643,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2656,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:35:04</t>
+          <t>Última actualización: 10:15:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2922,12 +3997,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:35:04</t>
+          <t>10:15:20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10:19</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2936,7 +4011,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2952,20 +4027,170 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:35:04</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>10:22</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>107</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>29</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>63</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>111</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:15:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>114</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4000
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:15:20</t>
+          <t>Última actualización: 12:27:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 109</t>
+          <t>Total filas: 141</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3190,6 +3190,806 @@
         <v>117</v>
       </c>
       <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>5</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>6</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>10</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>11</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>11</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>13</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>14</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>21</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>22</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>23</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>30</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>33</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>43</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>45</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>50</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>54</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>57</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>57</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>69</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>74</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>81</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>86</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>87</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>90</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>93</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>98</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>99</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>105</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>110</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>111</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>114</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3206,7 +4006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3219,14 +4019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:15:20</t>
+          <t>Última actualización: 12:27:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3702,6 +4502,56 @@
         <v>106</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>57</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>99</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3718,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3731,14 +4581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:15:20</t>
+          <t>Última actualización: 12:27:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4191,6 +5041,131 @@
       <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>31</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>44</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>47</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>60</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:27:42</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>77</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4001
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:27:42</t>
+          <t>Última actualización: 13:58:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 141</t>
+          <t>Total filas: 169</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>14:06</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>99</v>
+        <v>4</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>14:12</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>105</v>
+        <v>7</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:06</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>110</v>
+        <v>8</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>111</v>
+        <v>13</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,23 +3973,723 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>14:12</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>14</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>19</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>19</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>20</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>21</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
           <t>14:21</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C151" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D146" t="n">
-        <v>114</v>
-      </c>
-      <c r="E146" t="inlineStr">
+      <c r="D151" t="n">
+        <v>23</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>29</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>32</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>35</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>37</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>43</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>44</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>49</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>56</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>63</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>63</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>65</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>71</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>15:17</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>79</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>80</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>83</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>84</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>88</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>92</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>95</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>102</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>103</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>107</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>111</v>
+      </c>
+      <c r="E174" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4006,7 +4706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4019,14 +4719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:27:42</t>
+          <t>Última actualización: 13:58:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4535,7 +5235,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:27:42</t>
+          <t>13:58:39</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4549,9 +5249,134 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>32</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>63</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>107</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4568,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4581,14 +5406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:27:42</t>
+          <t>Última actualización: 13:58:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5166,6 +5991,81 @@
       <c r="E27" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>12</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>70</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>97</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4002
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:40</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 169</t>
+          <t>Total filas: 200</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>92</v>
+        <v>4</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>102</v>
+        <v>9</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>103</v>
+        <v>12</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>107</v>
+        <v>15</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,23 +4673,798 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>22</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>23</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>26</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
           <t>13:58:39</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>107</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>29</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>13:58:39</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
         <is>
           <t>15:49</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
+      <c r="C179" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D174" t="n">
+      <c r="D179" t="n">
         <v>111</v>
       </c>
-      <c r="E174" t="inlineStr">
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>40</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>42</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>42</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>47</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>48</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>52</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>56</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>62</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>63</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>63</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>69</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>16:28</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>70</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>76</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>79</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>16:39</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>81</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>82</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>86</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>87</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>16:49</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>91</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>97</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>97</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>100</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>101</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>101</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>111</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>112</v>
+      </c>
+      <c r="E205" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4706,7 +5481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4719,14 +5494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:40</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5335,7 +6110,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5349,7 +6124,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5360,23 +6135,123 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>26</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>13:58:39</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>107</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>86</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>97</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>112</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5393,7 +6268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5406,14 +6281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:40</t>
+          <t>Última actualización: 15:18:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6922,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:58:39</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6061,9 +6936,109 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>41</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>86</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>94</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>116</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4003
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 16:57:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 200</t>
+          <t>Total filas: 231</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,23 +5448,798 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>3</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>7</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>8</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>10</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>12</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
           <t>17:10</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C210" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D205" t="n">
-        <v>112</v>
-      </c>
-      <c r="E205" t="inlineStr">
+      <c r="D210" t="n">
+        <v>13</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>13</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>18</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>17:18</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>21</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>17:20</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>23</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>25</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>27</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>17:26</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>29</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>34</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>36</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>38</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>43</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>50</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>55</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>59</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>63</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>68</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>18:09</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>72</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>79</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>87</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>92</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>94</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>103</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>104</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>109</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>111</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>118</v>
+      </c>
+      <c r="E236" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5481,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5494,14 +6269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 16:57:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6235,7 +7010,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6249,9 +7024,84 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>112</v>
+        <v>13</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>104</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>109</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>111</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6268,7 +7118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6281,14 +7131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:18:44</t>
+          <t>Última actualización: 16:57:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7872,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7036,11 +7886,111 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>116</v>
+        <v>17</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>33</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>104</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>112</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>16:57:44</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>117</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4004
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:44</t>
+          <t>Última actualización: 18:01:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 231</t>
+          <t>Total filas: 252</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>18:09</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>79</v>
+        <v>4</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6053,16 +6053,16 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:09</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>18:29</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>103</v>
+        <v>16</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>104</v>
+        <v>16</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>111</v>
+        <v>22</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,23 +6223,548 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>23</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
           <t>16:57:44</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>92</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>29</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>30</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>39</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>40</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>45</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>47</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>18:52</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>51</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
         <is>
           <t>18:55</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C245" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D236" t="n">
-        <v>118</v>
-      </c>
-      <c r="E236" t="inlineStr">
+      <c r="D245" t="n">
+        <v>54</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>18:58</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>57</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>63</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>64</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>19:09</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>68</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>73</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>76</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>77</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>79</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>86</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>88</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>98</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>104</v>
+      </c>
+      <c r="E257" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6256,7 +6781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6269,14 +6794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:44</t>
+          <t>Última actualización: 18:01:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7560,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7049,7 +7574,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7060,7 +7585,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7074,7 +7599,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>109</v>
+        <v>45</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7085,7 +7610,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7099,9 +7624,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>111</v>
+        <v>47</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>76</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7131,7 +7681,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:44</t>
+          <t>Última actualización: 18:01:48</t>
         </is>
       </c>
     </row>
@@ -7922,7 +8472,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7936,7 +8486,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7947,7 +8497,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7961,7 +8511,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>112</v>
+        <v>48</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7972,7 +8522,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7986,7 +8536,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>117</v>
+        <v>53</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4005
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E257"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:48</t>
+          <t>Última actualización: 19:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 252</t>
+          <t>Total filas: 276</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6073,7 +6073,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>18:01:48</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -6083,11 +6083,11 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>18:01:48</t>
+          <t>19:17:09</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6678,16 +6678,16 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>18:01:48</t>
+          <t>19:17:09</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>18:01:48</t>
+          <t>19:17:09</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>19:39</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>98</v>
+        <v>4</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6753,18 +6753,618 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>86</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>11</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>19:29</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>88</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>13</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>22</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>18:01:48</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr">
+      <c r="C262" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D257" t="n">
+      <c r="D262" t="n">
         <v>104</v>
       </c>
-      <c r="E257" t="inlineStr">
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>29</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>30</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>36</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>45</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>49</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>49</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>49</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>20:13</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>56</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>61</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>61</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>64</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>71</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>76</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>82</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>85</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>91</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>97</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>100</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>21:13</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>116</v>
+      </c>
+      <c r="E281" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6781,7 +7381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6794,14 +7394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:48</t>
+          <t>Última actualización: 19:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7652,6 +8252,106 @@
         <v>76</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>76</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>85</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:48</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>91</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7668,7 +8368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7681,14 +8381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:48</t>
+          <t>Última actualización: 19:17:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -8541,6 +9241,106 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>61</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:28</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>84</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19:17:09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:08</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>111</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4006
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:17:10</t>
+          <t>Última actualización: 20:18:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 276</t>
+          <t>Total filas: 289</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D119" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7133,7 +7133,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7278,16 +7278,16 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>20:48</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>97</v>
+        <v>24</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:48</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,23 +7348,348 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>32</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>34</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>36</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>39</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>48</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
           <t>21:13</t>
         </is>
       </c>
-      <c r="C281" t="inlineStr">
+      <c r="C286" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D281" t="n">
-        <v>116</v>
-      </c>
-      <c r="E281" t="inlineStr">
+      <c r="D286" t="n">
+        <v>55</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>62</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>63</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>72</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>75</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>78</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>94</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>103</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>111</v>
+      </c>
+      <c r="E294" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7394,7 +7719,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:17:10</t>
+          <t>Última actualización: 20:18:10</t>
         </is>
       </c>
     </row>
@@ -7595,7 +7920,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -7620,7 +7945,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -8285,7 +8610,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -8299,7 +8624,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -8310,7 +8635,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8324,7 +8649,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -8335,7 +8660,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8349,7 +8674,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8368,7 +8693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8381,14 +8706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:17:10</t>
+          <t>Última actualización: 20:18:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9247,7 +9572,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9261,7 +9586,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -9272,7 +9597,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -9286,7 +9611,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -9297,7 +9622,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9311,7 +9636,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9322,7 +9647,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>20:18:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9336,11 +9661,36 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>114</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4007
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-05.xlsx
+++ b/data/horarios-141-2026-08-05.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E294"/>
+  <dimension ref="A1:E312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:10</t>
+          <t>Última actualización: 21:11:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 289</t>
+          <t>Total filas: 307</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>16:57:44</t>
+          <t>15:18:44</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>15:18:44</t>
+          <t>16:57:44</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5433,11 +5433,11 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>101</v>
+        <v>2</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>18:01:48</t>
+          <t>19:17:09</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>19:17:09</t>
+          <t>18:01:48</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>1</v>
+        <v>77</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7473,12 +7473,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>20:18:10</t>
+          <t>21:11:50</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7503,16 +7503,16 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>20:18:10</t>
+          <t>21:11:50</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:18</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>20:18:10</t>
+          <t>21:11:50</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:19</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>72</v>
+        <v>8</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>20:18:10</t>
+          <t>21:11:50</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>75</v>
+        <v>9</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7603,16 +7603,16 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7628,16 +7628,16 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7653,16 +7653,16 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>22:01</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,23 +7673,473 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>21</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>21</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
           <t>20:18:10</t>
         </is>
       </c>
-      <c r="B294" t="inlineStr">
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>75</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>24</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>78</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>94</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>49</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>103</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>57</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20:18:10</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
         <is>
           <t>22:09</t>
         </is>
       </c>
-      <c r="C294" t="inlineStr">
+      <c r="C303" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D294" t="n">
+      <c r="D303" t="n">
         <v>111</v>
       </c>
-      <c r="E294" t="inlineStr">
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>69</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>71</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>22:24</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>73</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>80</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>87</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>22:50</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>99</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>22:53</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>102</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>106</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>116</v>
+      </c>
+      <c r="E312" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7706,7 +8156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7719,14 +8169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:10</t>
+          <t>Última actualización: 21:11:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -8677,6 +9127,31 @@
         <v>30</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>106</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8693,7 +9168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8706,14 +9181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:18:10</t>
+          <t>Última actualización: 21:11:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -9672,23 +10147,73 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:18:10</t>
+          <t>21:11:50</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>21:57</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>46</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>22:12</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>114</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>61</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>21:11:50</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>70</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>